<commit_message>
Add DOCX in original Micro Session Planner format with colour-highlighted additions
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/session_plan/Revised_Micro_Session_Plan_DBMS_PLM_ORIGINAL_FORMAT.xlsx
+++ b/session_plan/Revised_Micro_Session_Plan_DBMS_PLM_ORIGINAL_FORMAT.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Micro Session Planner" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Micro Session Planner" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Micro Session Planner'!$11:$11</definedName>

</xml_diff>